<commit_message>
Economics + AI working
</commit_message>
<xml_diff>
--- a/outputs/economics_views_by_indicator.xlsx
+++ b/outputs/economics_views_by_indicator.xlsx
@@ -11,10 +11,13 @@
     <sheet name="consumer_confidence_index" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="gdp_current_prices" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="gdp_per_capita_current_prices" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="inflation_average_consumer_pric" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="population" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="real_gdp_growth_percent" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="unemployment_rate" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="household_disposable_income" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="inflation_average_consumer_pric" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="population" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="real_gdp_growth_percent" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="unemployment_rate" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="unemployment_rate_25_74_total" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="unemployment_rate_under_25_tota" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -420,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F361"/>
+  <dimension ref="A1:F454"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9453,6 +9456,2762 @@
         <is>
           <t>index</t>
         </is>
+      </c>
+    </row>
+    <row r="362">
+      <c r="A362" t="inlineStr">
+        <is>
+          <t>FR</t>
+        </is>
+      </c>
+      <c r="B362" t="inlineStr">
+        <is>
+          <t>household_disposable_income</t>
+        </is>
+      </c>
+      <c r="C362" t="n">
+        <v>2018</v>
+      </c>
+      <c r="D362" t="inlineStr"/>
+      <c r="E362" t="n">
+        <v>26257.1585330353</v>
+      </c>
+      <c r="F362" t="inlineStr">
+        <is>
+          <t>usd_dollars_per_person_PPP</t>
+        </is>
+      </c>
+    </row>
+    <row r="363">
+      <c r="A363" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="B363" t="inlineStr">
+        <is>
+          <t>household_disposable_income</t>
+        </is>
+      </c>
+      <c r="C363" t="n">
+        <v>2017</v>
+      </c>
+      <c r="D363" t="inlineStr"/>
+      <c r="E363" t="n">
+        <v>22141.1356335517</v>
+      </c>
+      <c r="F363" t="inlineStr">
+        <is>
+          <t>usd_dollars_per_person_PPP</t>
+        </is>
+      </c>
+    </row>
+    <row r="364">
+      <c r="A364" t="inlineStr">
+        <is>
+          <t>FR</t>
+        </is>
+      </c>
+      <c r="B364" t="inlineStr">
+        <is>
+          <t>household_disposable_income</t>
+        </is>
+      </c>
+      <c r="C364" t="n">
+        <v>2020</v>
+      </c>
+      <c r="D364" t="inlineStr"/>
+      <c r="E364" t="n">
+        <v>28877.5207135287</v>
+      </c>
+      <c r="F364" t="inlineStr">
+        <is>
+          <t>usd_dollars_per_person_PPP</t>
+        </is>
+      </c>
+    </row>
+    <row r="365">
+      <c r="A365" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="B365" t="inlineStr">
+        <is>
+          <t>household_disposable_income</t>
+        </is>
+      </c>
+      <c r="C365" t="n">
+        <v>2016</v>
+      </c>
+      <c r="D365" t="inlineStr"/>
+      <c r="E365" t="n">
+        <v>30246.5082874666</v>
+      </c>
+      <c r="F365" t="inlineStr">
+        <is>
+          <t>usd_dollars_per_person_PPP</t>
+        </is>
+      </c>
+    </row>
+    <row r="366">
+      <c r="A366" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="B366" t="inlineStr">
+        <is>
+          <t>household_disposable_income</t>
+        </is>
+      </c>
+      <c r="C366" t="n">
+        <v>2019</v>
+      </c>
+      <c r="D366" t="inlineStr"/>
+      <c r="E366" t="n">
+        <v>35351.7793839047</v>
+      </c>
+      <c r="F366" t="inlineStr">
+        <is>
+          <t>usd_dollars_per_person_PPP</t>
+        </is>
+      </c>
+    </row>
+    <row r="367">
+      <c r="A367" t="inlineStr">
+        <is>
+          <t>FR</t>
+        </is>
+      </c>
+      <c r="B367" t="inlineStr">
+        <is>
+          <t>household_disposable_income</t>
+        </is>
+      </c>
+      <c r="C367" t="n">
+        <v>2019</v>
+      </c>
+      <c r="D367" t="inlineStr"/>
+      <c r="E367" t="n">
+        <v>28146.378960002</v>
+      </c>
+      <c r="F367" t="inlineStr">
+        <is>
+          <t>usd_dollars_per_person_PPP</t>
+        </is>
+      </c>
+    </row>
+    <row r="368">
+      <c r="A368" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="B368" t="inlineStr">
+        <is>
+          <t>household_disposable_income</t>
+        </is>
+      </c>
+      <c r="C368" t="n">
+        <v>2018</v>
+      </c>
+      <c r="D368" t="inlineStr"/>
+      <c r="E368" t="n">
+        <v>22663.3314861856</v>
+      </c>
+      <c r="F368" t="inlineStr">
+        <is>
+          <t>usd_dollars_per_person_PPP</t>
+        </is>
+      </c>
+    </row>
+    <row r="369">
+      <c r="A369" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="B369" t="inlineStr">
+        <is>
+          <t>household_disposable_income</t>
+        </is>
+      </c>
+      <c r="C369" t="n">
+        <v>2017</v>
+      </c>
+      <c r="D369" t="inlineStr"/>
+      <c r="E369" t="n">
+        <v>31570.8974904355</v>
+      </c>
+      <c r="F369" t="inlineStr">
+        <is>
+          <t>usd_dollars_per_person_PPP</t>
+        </is>
+      </c>
+    </row>
+    <row r="370">
+      <c r="A370" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="B370" t="inlineStr">
+        <is>
+          <t>household_disposable_income</t>
+        </is>
+      </c>
+      <c r="C370" t="n">
+        <v>2020</v>
+      </c>
+      <c r="D370" t="inlineStr"/>
+      <c r="E370" t="n">
+        <v>23782.4678049223</v>
+      </c>
+      <c r="F370" t="inlineStr">
+        <is>
+          <t>usd_dollars_per_person_PPP</t>
+        </is>
+      </c>
+    </row>
+    <row r="371">
+      <c r="A371" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="B371" t="inlineStr">
+        <is>
+          <t>household_disposable_income</t>
+        </is>
+      </c>
+      <c r="C371" t="n">
+        <v>2020</v>
+      </c>
+      <c r="D371" t="inlineStr"/>
+      <c r="E371" t="n">
+        <v>36071.5163052037</v>
+      </c>
+      <c r="F371" t="inlineStr">
+        <is>
+          <t>usd_dollars_per_person_PPP</t>
+        </is>
+      </c>
+    </row>
+    <row r="372">
+      <c r="A372" t="inlineStr">
+        <is>
+          <t>FR</t>
+        </is>
+      </c>
+      <c r="B372" t="inlineStr">
+        <is>
+          <t>household_disposable_income</t>
+        </is>
+      </c>
+      <c r="C372" t="n">
+        <v>2016</v>
+      </c>
+      <c r="D372" t="inlineStr"/>
+      <c r="E372" t="n">
+        <v>24924.9379154554</v>
+      </c>
+      <c r="F372" t="inlineStr">
+        <is>
+          <t>usd_dollars_per_person_PPP</t>
+        </is>
+      </c>
+    </row>
+    <row r="373">
+      <c r="A373" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="B373" t="inlineStr">
+        <is>
+          <t>household_disposable_income</t>
+        </is>
+      </c>
+      <c r="C373" t="n">
+        <v>2024</v>
+      </c>
+      <c r="D373" t="inlineStr"/>
+      <c r="E373" t="n">
+        <v>35161.9297398487</v>
+      </c>
+      <c r="F373" t="inlineStr">
+        <is>
+          <t>usd_dollars_per_person_PPP</t>
+        </is>
+      </c>
+    </row>
+    <row r="374">
+      <c r="A374" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="B374" t="inlineStr">
+        <is>
+          <t>household_disposable_income</t>
+        </is>
+      </c>
+      <c r="C374" t="n">
+        <v>2024</v>
+      </c>
+      <c r="D374" t="inlineStr"/>
+      <c r="E374" t="n">
+        <v>47685.3791601533</v>
+      </c>
+      <c r="F374" t="inlineStr">
+        <is>
+          <t>usd_dollars_per_person_PPP</t>
+        </is>
+      </c>
+    </row>
+    <row r="375">
+      <c r="A375" t="inlineStr">
+        <is>
+          <t>FR</t>
+        </is>
+      </c>
+      <c r="B375" t="inlineStr">
+        <is>
+          <t>household_disposable_income</t>
+        </is>
+      </c>
+      <c r="C375" t="n">
+        <v>2024</v>
+      </c>
+      <c r="D375" t="inlineStr"/>
+      <c r="E375" t="n">
+        <v>39420.8018012013</v>
+      </c>
+      <c r="F375" t="inlineStr">
+        <is>
+          <t>usd_dollars_per_person_PPP</t>
+        </is>
+      </c>
+    </row>
+    <row r="376">
+      <c r="A376" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="B376" t="inlineStr">
+        <is>
+          <t>household_disposable_income</t>
+        </is>
+      </c>
+      <c r="C376" t="n">
+        <v>2023</v>
+      </c>
+      <c r="D376" t="inlineStr"/>
+      <c r="E376" t="n">
+        <v>33453.2943583124</v>
+      </c>
+      <c r="F376" t="inlineStr">
+        <is>
+          <t>usd_dollars_per_person_PPP</t>
+        </is>
+      </c>
+    </row>
+    <row r="377">
+      <c r="A377" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="B377" t="inlineStr">
+        <is>
+          <t>household_disposable_income</t>
+        </is>
+      </c>
+      <c r="C377" t="n">
+        <v>2023</v>
+      </c>
+      <c r="D377" t="inlineStr"/>
+      <c r="E377" t="n">
+        <v>45926.6267519884</v>
+      </c>
+      <c r="F377" t="inlineStr">
+        <is>
+          <t>usd_dollars_per_person_PPP</t>
+        </is>
+      </c>
+    </row>
+    <row r="378">
+      <c r="A378" t="inlineStr">
+        <is>
+          <t>FR</t>
+        </is>
+      </c>
+      <c r="B378" t="inlineStr">
+        <is>
+          <t>household_disposable_income</t>
+        </is>
+      </c>
+      <c r="C378" t="n">
+        <v>2023</v>
+      </c>
+      <c r="D378" t="inlineStr"/>
+      <c r="E378" t="n">
+        <v>37582.228371007</v>
+      </c>
+      <c r="F378" t="inlineStr">
+        <is>
+          <t>usd_dollars_per_person_PPP</t>
+        </is>
+      </c>
+    </row>
+    <row r="379">
+      <c r="A379" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="B379" t="inlineStr">
+        <is>
+          <t>household_disposable_income</t>
+        </is>
+      </c>
+      <c r="C379" t="n">
+        <v>2022</v>
+      </c>
+      <c r="D379" t="inlineStr"/>
+      <c r="E379" t="n">
+        <v>42501.3770918378</v>
+      </c>
+      <c r="F379" t="inlineStr">
+        <is>
+          <t>usd_dollars_per_person_PPP</t>
+        </is>
+      </c>
+    </row>
+    <row r="380">
+      <c r="A380" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="B380" t="inlineStr">
+        <is>
+          <t>household_disposable_income</t>
+        </is>
+      </c>
+      <c r="C380" t="n">
+        <v>2022</v>
+      </c>
+      <c r="D380" t="inlineStr"/>
+      <c r="E380" t="n">
+        <v>28726.1264569898</v>
+      </c>
+      <c r="F380" t="inlineStr">
+        <is>
+          <t>usd_dollars_per_person_PPP</t>
+        </is>
+      </c>
+    </row>
+    <row r="381">
+      <c r="A381" t="inlineStr">
+        <is>
+          <t>FR</t>
+        </is>
+      </c>
+      <c r="B381" t="inlineStr">
+        <is>
+          <t>household_disposable_income</t>
+        </is>
+      </c>
+      <c r="C381" t="n">
+        <v>2022</v>
+      </c>
+      <c r="D381" t="inlineStr"/>
+      <c r="E381" t="n">
+        <v>33737.7298976999</v>
+      </c>
+      <c r="F381" t="inlineStr">
+        <is>
+          <t>usd_dollars_per_person_PPP</t>
+        </is>
+      </c>
+    </row>
+    <row r="382">
+      <c r="A382" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="B382" t="inlineStr">
+        <is>
+          <t>household_disposable_income</t>
+        </is>
+      </c>
+      <c r="C382" t="n">
+        <v>2021</v>
+      </c>
+      <c r="D382" t="inlineStr"/>
+      <c r="E382" t="n">
+        <v>26175.863403135</v>
+      </c>
+      <c r="F382" t="inlineStr">
+        <is>
+          <t>usd_dollars_per_person_PPP</t>
+        </is>
+      </c>
+    </row>
+    <row r="383">
+      <c r="A383" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="B383" t="inlineStr">
+        <is>
+          <t>household_disposable_income</t>
+        </is>
+      </c>
+      <c r="C383" t="n">
+        <v>2021</v>
+      </c>
+      <c r="D383" t="inlineStr"/>
+      <c r="E383" t="n">
+        <v>37802.9092037468</v>
+      </c>
+      <c r="F383" t="inlineStr">
+        <is>
+          <t>usd_dollars_per_person_PPP</t>
+        </is>
+      </c>
+    </row>
+    <row r="384">
+      <c r="A384" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="B384" t="inlineStr">
+        <is>
+          <t>household_disposable_income</t>
+        </is>
+      </c>
+      <c r="C384" t="n">
+        <v>2019</v>
+      </c>
+      <c r="D384" t="inlineStr"/>
+      <c r="E384" t="n">
+        <v>24582.9902204603</v>
+      </c>
+      <c r="F384" t="inlineStr">
+        <is>
+          <t>usd_dollars_per_person_PPP</t>
+        </is>
+      </c>
+    </row>
+    <row r="385">
+      <c r="A385" t="inlineStr">
+        <is>
+          <t>FR</t>
+        </is>
+      </c>
+      <c r="B385" t="inlineStr">
+        <is>
+          <t>household_disposable_income</t>
+        </is>
+      </c>
+      <c r="C385" t="n">
+        <v>2017</v>
+      </c>
+      <c r="D385" t="inlineStr"/>
+      <c r="E385" t="n">
+        <v>25436.327661389</v>
+      </c>
+      <c r="F385" t="inlineStr">
+        <is>
+          <t>usd_dollars_per_person_PPP</t>
+        </is>
+      </c>
+    </row>
+    <row r="386">
+      <c r="A386" t="inlineStr">
+        <is>
+          <t>FR</t>
+        </is>
+      </c>
+      <c r="B386" t="inlineStr">
+        <is>
+          <t>household_disposable_income</t>
+        </is>
+      </c>
+      <c r="C386" t="n">
+        <v>2021</v>
+      </c>
+      <c r="D386" t="inlineStr"/>
+      <c r="E386" t="n">
+        <v>30167.6571699568</v>
+      </c>
+      <c r="F386" t="inlineStr">
+        <is>
+          <t>usd_dollars_per_person_PPP</t>
+        </is>
+      </c>
+    </row>
+    <row r="387">
+      <c r="A387" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="B387" t="inlineStr">
+        <is>
+          <t>household_disposable_income</t>
+        </is>
+      </c>
+      <c r="C387" t="n">
+        <v>2018</v>
+      </c>
+      <c r="D387" t="inlineStr"/>
+      <c r="E387" t="n">
+        <v>33615.1802446285</v>
+      </c>
+      <c r="F387" t="inlineStr">
+        <is>
+          <t>usd_dollars_per_person_PPP</t>
+        </is>
+      </c>
+    </row>
+    <row r="388">
+      <c r="A388" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="B388" t="inlineStr">
+        <is>
+          <t>household_disposable_income</t>
+        </is>
+      </c>
+      <c r="C388" t="n">
+        <v>2016</v>
+      </c>
+      <c r="D388" t="inlineStr"/>
+      <c r="E388" t="n">
+        <v>21291.8728491478</v>
+      </c>
+      <c r="F388" t="inlineStr">
+        <is>
+          <t>usd_dollars_per_person_PPP</t>
+        </is>
+      </c>
+    </row>
+    <row r="389">
+      <c r="A389" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="B389" t="inlineStr">
+        <is>
+          <t>unemployment_rate_under_25_total</t>
+        </is>
+      </c>
+      <c r="C389" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D389" t="n">
+        <v>2</v>
+      </c>
+      <c r="E389" t="n">
+        <v>26.3</v>
+      </c>
+      <c r="F389" t="inlineStr">
+        <is>
+          <t>PC_ACT</t>
+        </is>
+      </c>
+    </row>
+    <row r="390">
+      <c r="A390" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="B390" t="inlineStr">
+        <is>
+          <t>unemployment_rate_under_25_total</t>
+        </is>
+      </c>
+      <c r="C390" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D390" t="n">
+        <v>3</v>
+      </c>
+      <c r="E390" t="n">
+        <v>26.2</v>
+      </c>
+      <c r="F390" t="inlineStr">
+        <is>
+          <t>PC_ACT</t>
+        </is>
+      </c>
+    </row>
+    <row r="391">
+      <c r="A391" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="B391" t="inlineStr">
+        <is>
+          <t>unemployment_rate_under_25_total</t>
+        </is>
+      </c>
+      <c r="C391" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D391" t="n">
+        <v>4</v>
+      </c>
+      <c r="E391" t="n">
+        <v>24.9</v>
+      </c>
+      <c r="F391" t="inlineStr">
+        <is>
+          <t>PC_ACT</t>
+        </is>
+      </c>
+    </row>
+    <row r="392">
+      <c r="A392" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="B392" t="inlineStr">
+        <is>
+          <t>unemployment_rate_under_25_total</t>
+        </is>
+      </c>
+      <c r="C392" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D392" t="n">
+        <v>5</v>
+      </c>
+      <c r="E392" t="n">
+        <v>24.8</v>
+      </c>
+      <c r="F392" t="inlineStr">
+        <is>
+          <t>PC_ACT</t>
+        </is>
+      </c>
+    </row>
+    <row r="393">
+      <c r="A393" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="B393" t="inlineStr">
+        <is>
+          <t>unemployment_rate_under_25_total</t>
+        </is>
+      </c>
+      <c r="C393" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D393" t="n">
+        <v>6</v>
+      </c>
+      <c r="E393" t="n">
+        <v>24.6</v>
+      </c>
+      <c r="F393" t="inlineStr">
+        <is>
+          <t>PC_ACT</t>
+        </is>
+      </c>
+    </row>
+    <row r="394">
+      <c r="A394" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="B394" t="inlineStr">
+        <is>
+          <t>unemployment_rate_under_25_total</t>
+        </is>
+      </c>
+      <c r="C394" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D394" t="n">
+        <v>7</v>
+      </c>
+      <c r="E394" t="n">
+        <v>24.9</v>
+      </c>
+      <c r="F394" t="inlineStr">
+        <is>
+          <t>PC_ACT</t>
+        </is>
+      </c>
+    </row>
+    <row r="395">
+      <c r="A395" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="B395" t="inlineStr">
+        <is>
+          <t>unemployment_rate_under_25_total</t>
+        </is>
+      </c>
+      <c r="C395" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D395" t="n">
+        <v>8</v>
+      </c>
+      <c r="E395" t="n">
+        <v>24.8</v>
+      </c>
+      <c r="F395" t="inlineStr">
+        <is>
+          <t>PC_ACT</t>
+        </is>
+      </c>
+    </row>
+    <row r="396">
+      <c r="A396" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="B396" t="inlineStr">
+        <is>
+          <t>unemployment_rate_under_25_total</t>
+        </is>
+      </c>
+      <c r="C396" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D396" t="n">
+        <v>9</v>
+      </c>
+      <c r="E396" t="n">
+        <v>24.6</v>
+      </c>
+      <c r="F396" t="inlineStr">
+        <is>
+          <t>PC_ACT</t>
+        </is>
+      </c>
+    </row>
+    <row r="397">
+      <c r="A397" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="B397" t="inlineStr">
+        <is>
+          <t>unemployment_rate_under_25_total</t>
+        </is>
+      </c>
+      <c r="C397" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D397" t="n">
+        <v>10</v>
+      </c>
+      <c r="E397" t="n">
+        <v>24.1</v>
+      </c>
+      <c r="F397" t="inlineStr">
+        <is>
+          <t>PC_ACT</t>
+        </is>
+      </c>
+    </row>
+    <row r="398">
+      <c r="A398" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="B398" t="inlineStr">
+        <is>
+          <t>unemployment_rate_under_25_total</t>
+        </is>
+      </c>
+      <c r="C398" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D398" t="n">
+        <v>11</v>
+      </c>
+      <c r="E398" t="n">
+        <v>23.6</v>
+      </c>
+      <c r="F398" t="inlineStr">
+        <is>
+          <t>PC_ACT</t>
+        </is>
+      </c>
+    </row>
+    <row r="399">
+      <c r="A399" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="B399" t="inlineStr">
+        <is>
+          <t>unemployment_rate_under_25_total</t>
+        </is>
+      </c>
+      <c r="C399" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D399" t="n">
+        <v>12</v>
+      </c>
+      <c r="E399" t="n">
+        <v>23.4</v>
+      </c>
+      <c r="F399" t="inlineStr">
+        <is>
+          <t>PC_ACT</t>
+        </is>
+      </c>
+    </row>
+    <row r="400">
+      <c r="A400" t="inlineStr">
+        <is>
+          <t>FR</t>
+        </is>
+      </c>
+      <c r="B400" t="inlineStr">
+        <is>
+          <t>unemployment_rate_under_25_total</t>
+        </is>
+      </c>
+      <c r="C400" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D400" t="n">
+        <v>2</v>
+      </c>
+      <c r="E400" t="n">
+        <v>19.8</v>
+      </c>
+      <c r="F400" t="inlineStr">
+        <is>
+          <t>PC_ACT</t>
+        </is>
+      </c>
+    </row>
+    <row r="401">
+      <c r="A401" t="inlineStr">
+        <is>
+          <t>FR</t>
+        </is>
+      </c>
+      <c r="B401" t="inlineStr">
+        <is>
+          <t>unemployment_rate_under_25_total</t>
+        </is>
+      </c>
+      <c r="C401" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D401" t="n">
+        <v>3</v>
+      </c>
+      <c r="E401" t="n">
+        <v>19</v>
+      </c>
+      <c r="F401" t="inlineStr">
+        <is>
+          <t>PC_ACT</t>
+        </is>
+      </c>
+    </row>
+    <row r="402">
+      <c r="A402" t="inlineStr">
+        <is>
+          <t>FR</t>
+        </is>
+      </c>
+      <c r="B402" t="inlineStr">
+        <is>
+          <t>unemployment_rate_under_25_total</t>
+        </is>
+      </c>
+      <c r="C402" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D402" t="n">
+        <v>4</v>
+      </c>
+      <c r="E402" t="n">
+        <v>18.9</v>
+      </c>
+      <c r="F402" t="inlineStr">
+        <is>
+          <t>PC_ACT</t>
+        </is>
+      </c>
+    </row>
+    <row r="403">
+      <c r="A403" t="inlineStr">
+        <is>
+          <t>FR</t>
+        </is>
+      </c>
+      <c r="B403" t="inlineStr">
+        <is>
+          <t>unemployment_rate_under_25_total</t>
+        </is>
+      </c>
+      <c r="C403" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D403" t="n">
+        <v>5</v>
+      </c>
+      <c r="E403" t="n">
+        <v>19.1</v>
+      </c>
+      <c r="F403" t="inlineStr">
+        <is>
+          <t>PC_ACT</t>
+        </is>
+      </c>
+    </row>
+    <row r="404">
+      <c r="A404" t="inlineStr">
+        <is>
+          <t>FR</t>
+        </is>
+      </c>
+      <c r="B404" t="inlineStr">
+        <is>
+          <t>unemployment_rate_under_25_total</t>
+        </is>
+      </c>
+      <c r="C404" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D404" t="n">
+        <v>6</v>
+      </c>
+      <c r="E404" t="n">
+        <v>18.8</v>
+      </c>
+      <c r="F404" t="inlineStr">
+        <is>
+          <t>PC_ACT</t>
+        </is>
+      </c>
+    </row>
+    <row r="405">
+      <c r="A405" t="inlineStr">
+        <is>
+          <t>FR</t>
+        </is>
+      </c>
+      <c r="B405" t="inlineStr">
+        <is>
+          <t>unemployment_rate_under_25_total</t>
+        </is>
+      </c>
+      <c r="C405" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D405" t="n">
+        <v>7</v>
+      </c>
+      <c r="E405" t="n">
+        <v>18.5</v>
+      </c>
+      <c r="F405" t="inlineStr">
+        <is>
+          <t>PC_ACT</t>
+        </is>
+      </c>
+    </row>
+    <row r="406">
+      <c r="A406" t="inlineStr">
+        <is>
+          <t>FR</t>
+        </is>
+      </c>
+      <c r="B406" t="inlineStr">
+        <is>
+          <t>unemployment_rate_under_25_total</t>
+        </is>
+      </c>
+      <c r="C406" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D406" t="n">
+        <v>8</v>
+      </c>
+      <c r="E406" t="n">
+        <v>18.6</v>
+      </c>
+      <c r="F406" t="inlineStr">
+        <is>
+          <t>PC_ACT</t>
+        </is>
+      </c>
+    </row>
+    <row r="407">
+      <c r="A407" t="inlineStr">
+        <is>
+          <t>FR</t>
+        </is>
+      </c>
+      <c r="B407" t="inlineStr">
+        <is>
+          <t>unemployment_rate_under_25_total</t>
+        </is>
+      </c>
+      <c r="C407" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D407" t="n">
+        <v>9</v>
+      </c>
+      <c r="E407" t="n">
+        <v>19</v>
+      </c>
+      <c r="F407" t="inlineStr">
+        <is>
+          <t>PC_ACT</t>
+        </is>
+      </c>
+    </row>
+    <row r="408">
+      <c r="A408" t="inlineStr">
+        <is>
+          <t>FR</t>
+        </is>
+      </c>
+      <c r="B408" t="inlineStr">
+        <is>
+          <t>unemployment_rate_under_25_total</t>
+        </is>
+      </c>
+      <c r="C408" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D408" t="n">
+        <v>10</v>
+      </c>
+      <c r="E408" t="n">
+        <v>18.9</v>
+      </c>
+      <c r="F408" t="inlineStr">
+        <is>
+          <t>PC_ACT</t>
+        </is>
+      </c>
+    </row>
+    <row r="409">
+      <c r="A409" t="inlineStr">
+        <is>
+          <t>FR</t>
+        </is>
+      </c>
+      <c r="B409" t="inlineStr">
+        <is>
+          <t>unemployment_rate_under_25_total</t>
+        </is>
+      </c>
+      <c r="C409" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D409" t="n">
+        <v>11</v>
+      </c>
+      <c r="E409" t="n">
+        <v>18.5</v>
+      </c>
+      <c r="F409" t="inlineStr">
+        <is>
+          <t>PC_ACT</t>
+        </is>
+      </c>
+    </row>
+    <row r="410">
+      <c r="A410" t="inlineStr">
+        <is>
+          <t>FR</t>
+        </is>
+      </c>
+      <c r="B410" t="inlineStr">
+        <is>
+          <t>unemployment_rate_under_25_total</t>
+        </is>
+      </c>
+      <c r="C410" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D410" t="n">
+        <v>12</v>
+      </c>
+      <c r="E410" t="n">
+        <v>18.1</v>
+      </c>
+      <c r="F410" t="inlineStr">
+        <is>
+          <t>PC_ACT</t>
+        </is>
+      </c>
+    </row>
+    <row r="411">
+      <c r="A411" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="B411" t="inlineStr">
+        <is>
+          <t>unemployment_rate_under_25_total</t>
+        </is>
+      </c>
+      <c r="C411" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D411" t="n">
+        <v>2</v>
+      </c>
+      <c r="E411" t="n">
+        <v>6.8</v>
+      </c>
+      <c r="F411" t="inlineStr">
+        <is>
+          <t>PC_ACT</t>
+        </is>
+      </c>
+    </row>
+    <row r="412">
+      <c r="A412" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="B412" t="inlineStr">
+        <is>
+          <t>unemployment_rate_under_25_total</t>
+        </is>
+      </c>
+      <c r="C412" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D412" t="n">
+        <v>3</v>
+      </c>
+      <c r="E412" t="n">
+        <v>6.8</v>
+      </c>
+      <c r="F412" t="inlineStr">
+        <is>
+          <t>PC_ACT</t>
+        </is>
+      </c>
+    </row>
+    <row r="413">
+      <c r="A413" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="B413" t="inlineStr">
+        <is>
+          <t>unemployment_rate_under_25_total</t>
+        </is>
+      </c>
+      <c r="C413" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D413" t="n">
+        <v>4</v>
+      </c>
+      <c r="E413" t="n">
+        <v>6.8</v>
+      </c>
+      <c r="F413" t="inlineStr">
+        <is>
+          <t>PC_ACT</t>
+        </is>
+      </c>
+    </row>
+    <row r="414">
+      <c r="A414" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="B414" t="inlineStr">
+        <is>
+          <t>unemployment_rate_under_25_total</t>
+        </is>
+      </c>
+      <c r="C414" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D414" t="n">
+        <v>5</v>
+      </c>
+      <c r="E414" t="n">
+        <v>6.8</v>
+      </c>
+      <c r="F414" t="inlineStr">
+        <is>
+          <t>PC_ACT</t>
+        </is>
+      </c>
+    </row>
+    <row r="415">
+      <c r="A415" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="B415" t="inlineStr">
+        <is>
+          <t>unemployment_rate_under_25_total</t>
+        </is>
+      </c>
+      <c r="C415" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D415" t="n">
+        <v>6</v>
+      </c>
+      <c r="E415" t="n">
+        <v>6.9</v>
+      </c>
+      <c r="F415" t="inlineStr">
+        <is>
+          <t>PC_ACT</t>
+        </is>
+      </c>
+    </row>
+    <row r="416">
+      <c r="A416" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="B416" t="inlineStr">
+        <is>
+          <t>unemployment_rate_under_25_total</t>
+        </is>
+      </c>
+      <c r="C416" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D416" t="n">
+        <v>7</v>
+      </c>
+      <c r="E416" t="n">
+        <v>6.9</v>
+      </c>
+      <c r="F416" t="inlineStr">
+        <is>
+          <t>PC_ACT</t>
+        </is>
+      </c>
+    </row>
+    <row r="417">
+      <c r="A417" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="B417" t="inlineStr">
+        <is>
+          <t>unemployment_rate_under_25_total</t>
+        </is>
+      </c>
+      <c r="C417" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D417" t="n">
+        <v>8</v>
+      </c>
+      <c r="E417" t="n">
+        <v>6.9</v>
+      </c>
+      <c r="F417" t="inlineStr">
+        <is>
+          <t>PC_ACT</t>
+        </is>
+      </c>
+    </row>
+    <row r="418">
+      <c r="A418" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="B418" t="inlineStr">
+        <is>
+          <t>unemployment_rate_under_25_total</t>
+        </is>
+      </c>
+      <c r="C418" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D418" t="n">
+        <v>9</v>
+      </c>
+      <c r="E418" t="n">
+        <v>6.9</v>
+      </c>
+      <c r="F418" t="inlineStr">
+        <is>
+          <t>PC_ACT</t>
+        </is>
+      </c>
+    </row>
+    <row r="419">
+      <c r="A419" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="B419" t="inlineStr">
+        <is>
+          <t>unemployment_rate_under_25_total</t>
+        </is>
+      </c>
+      <c r="C419" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D419" t="n">
+        <v>10</v>
+      </c>
+      <c r="E419" t="n">
+        <v>6.9</v>
+      </c>
+      <c r="F419" t="inlineStr">
+        <is>
+          <t>PC_ACT</t>
+        </is>
+      </c>
+    </row>
+    <row r="420">
+      <c r="A420" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="B420" t="inlineStr">
+        <is>
+          <t>unemployment_rate_under_25_total</t>
+        </is>
+      </c>
+      <c r="C420" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D420" t="n">
+        <v>11</v>
+      </c>
+      <c r="E420" t="n">
+        <v>6.8</v>
+      </c>
+      <c r="F420" t="inlineStr">
+        <is>
+          <t>PC_ACT</t>
+        </is>
+      </c>
+    </row>
+    <row r="421">
+      <c r="A421" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="B421" t="inlineStr">
+        <is>
+          <t>unemployment_rate_under_25_total</t>
+        </is>
+      </c>
+      <c r="C421" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D421" t="n">
+        <v>12</v>
+      </c>
+      <c r="E421" t="n">
+        <v>6.8</v>
+      </c>
+      <c r="F421" t="inlineStr">
+        <is>
+          <t>PC_ACT</t>
+        </is>
+      </c>
+    </row>
+    <row r="422">
+      <c r="A422" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="B422" t="inlineStr">
+        <is>
+          <t>unemployment_rate_25_74_total</t>
+        </is>
+      </c>
+      <c r="C422" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D422" t="n">
+        <v>2</v>
+      </c>
+      <c r="E422" t="n">
+        <v>9.6</v>
+      </c>
+      <c r="F422" t="inlineStr">
+        <is>
+          <t>PC_ACT</t>
+        </is>
+      </c>
+    </row>
+    <row r="423">
+      <c r="A423" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="B423" t="inlineStr">
+        <is>
+          <t>unemployment_rate_25_74_total</t>
+        </is>
+      </c>
+      <c r="C423" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D423" t="n">
+        <v>3</v>
+      </c>
+      <c r="E423" t="n">
+        <v>9.6</v>
+      </c>
+      <c r="F423" t="inlineStr">
+        <is>
+          <t>PC_ACT</t>
+        </is>
+      </c>
+    </row>
+    <row r="424">
+      <c r="A424" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="B424" t="inlineStr">
+        <is>
+          <t>unemployment_rate_25_74_total</t>
+        </is>
+      </c>
+      <c r="C424" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D424" t="n">
+        <v>4</v>
+      </c>
+      <c r="E424" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="F424" t="inlineStr">
+        <is>
+          <t>PC_ACT</t>
+        </is>
+      </c>
+    </row>
+    <row r="425">
+      <c r="A425" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="B425" t="inlineStr">
+        <is>
+          <t>unemployment_rate_25_74_total</t>
+        </is>
+      </c>
+      <c r="C425" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D425" t="n">
+        <v>5</v>
+      </c>
+      <c r="E425" t="n">
+        <v>9.4</v>
+      </c>
+      <c r="F425" t="inlineStr">
+        <is>
+          <t>PC_ACT</t>
+        </is>
+      </c>
+    </row>
+    <row r="426">
+      <c r="A426" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="B426" t="inlineStr">
+        <is>
+          <t>unemployment_rate_25_74_total</t>
+        </is>
+      </c>
+      <c r="C426" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D426" t="n">
+        <v>6</v>
+      </c>
+      <c r="E426" t="n">
+        <v>9.4</v>
+      </c>
+      <c r="F426" t="inlineStr">
+        <is>
+          <t>PC_ACT</t>
+        </is>
+      </c>
+    </row>
+    <row r="427">
+      <c r="A427" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="B427" t="inlineStr">
+        <is>
+          <t>unemployment_rate_25_74_total</t>
+        </is>
+      </c>
+      <c r="C427" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D427" t="n">
+        <v>7</v>
+      </c>
+      <c r="E427" t="n">
+        <v>9.4</v>
+      </c>
+      <c r="F427" t="inlineStr">
+        <is>
+          <t>PC_ACT</t>
+        </is>
+      </c>
+    </row>
+    <row r="428">
+      <c r="A428" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="B428" t="inlineStr">
+        <is>
+          <t>unemployment_rate_25_74_total</t>
+        </is>
+      </c>
+      <c r="C428" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D428" t="n">
+        <v>8</v>
+      </c>
+      <c r="E428" t="n">
+        <v>9.300000000000001</v>
+      </c>
+      <c r="F428" t="inlineStr">
+        <is>
+          <t>PC_ACT</t>
+        </is>
+      </c>
+    </row>
+    <row r="429">
+      <c r="A429" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="B429" t="inlineStr">
+        <is>
+          <t>unemployment_rate_25_74_total</t>
+        </is>
+      </c>
+      <c r="C429" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D429" t="n">
+        <v>9</v>
+      </c>
+      <c r="E429" t="n">
+        <v>9.300000000000001</v>
+      </c>
+      <c r="F429" t="inlineStr">
+        <is>
+          <t>PC_ACT</t>
+        </is>
+      </c>
+    </row>
+    <row r="430">
+      <c r="A430" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="B430" t="inlineStr">
+        <is>
+          <t>unemployment_rate_25_74_total</t>
+        </is>
+      </c>
+      <c r="C430" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D430" t="n">
+        <v>10</v>
+      </c>
+      <c r="E430" t="n">
+        <v>9.1</v>
+      </c>
+      <c r="F430" t="inlineStr">
+        <is>
+          <t>PC_ACT</t>
+        </is>
+      </c>
+    </row>
+    <row r="431">
+      <c r="A431" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="B431" t="inlineStr">
+        <is>
+          <t>unemployment_rate_25_74_total</t>
+        </is>
+      </c>
+      <c r="C431" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D431" t="n">
+        <v>11</v>
+      </c>
+      <c r="E431" t="n">
+        <v>9.1</v>
+      </c>
+      <c r="F431" t="inlineStr">
+        <is>
+          <t>PC_ACT</t>
+        </is>
+      </c>
+    </row>
+    <row r="432">
+      <c r="A432" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="B432" t="inlineStr">
+        <is>
+          <t>unemployment_rate_25_74_total</t>
+        </is>
+      </c>
+      <c r="C432" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D432" t="n">
+        <v>12</v>
+      </c>
+      <c r="E432" t="n">
+        <v>9</v>
+      </c>
+      <c r="F432" t="inlineStr">
+        <is>
+          <t>PC_ACT</t>
+        </is>
+      </c>
+    </row>
+    <row r="433">
+      <c r="A433" t="inlineStr">
+        <is>
+          <t>FR</t>
+        </is>
+      </c>
+      <c r="B433" t="inlineStr">
+        <is>
+          <t>unemployment_rate_25_74_total</t>
+        </is>
+      </c>
+      <c r="C433" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D433" t="n">
+        <v>2</v>
+      </c>
+      <c r="E433" t="n">
+        <v>6</v>
+      </c>
+      <c r="F433" t="inlineStr">
+        <is>
+          <t>PC_ACT</t>
+        </is>
+      </c>
+    </row>
+    <row r="434">
+      <c r="A434" t="inlineStr">
+        <is>
+          <t>FR</t>
+        </is>
+      </c>
+      <c r="B434" t="inlineStr">
+        <is>
+          <t>unemployment_rate_25_74_total</t>
+        </is>
+      </c>
+      <c r="C434" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D434" t="n">
+        <v>3</v>
+      </c>
+      <c r="E434" t="n">
+        <v>6.2</v>
+      </c>
+      <c r="F434" t="inlineStr">
+        <is>
+          <t>PC_ACT</t>
+        </is>
+      </c>
+    </row>
+    <row r="435">
+      <c r="A435" t="inlineStr">
+        <is>
+          <t>FR</t>
+        </is>
+      </c>
+      <c r="B435" t="inlineStr">
+        <is>
+          <t>unemployment_rate_25_74_total</t>
+        </is>
+      </c>
+      <c r="C435" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D435" t="n">
+        <v>4</v>
+      </c>
+      <c r="E435" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="F435" t="inlineStr">
+        <is>
+          <t>PC_ACT</t>
+        </is>
+      </c>
+    </row>
+    <row r="436">
+      <c r="A436" t="inlineStr">
+        <is>
+          <t>FR</t>
+        </is>
+      </c>
+      <c r="B436" t="inlineStr">
+        <is>
+          <t>unemployment_rate_25_74_total</t>
+        </is>
+      </c>
+      <c r="C436" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D436" t="n">
+        <v>5</v>
+      </c>
+      <c r="E436" t="n">
+        <v>6.2</v>
+      </c>
+      <c r="F436" t="inlineStr">
+        <is>
+          <t>PC_ACT</t>
+        </is>
+      </c>
+    </row>
+    <row r="437">
+      <c r="A437" t="inlineStr">
+        <is>
+          <t>FR</t>
+        </is>
+      </c>
+      <c r="B437" t="inlineStr">
+        <is>
+          <t>unemployment_rate_25_74_total</t>
+        </is>
+      </c>
+      <c r="C437" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D437" t="n">
+        <v>6</v>
+      </c>
+      <c r="E437" t="n">
+        <v>6.3</v>
+      </c>
+      <c r="F437" t="inlineStr">
+        <is>
+          <t>PC_ACT</t>
+        </is>
+      </c>
+    </row>
+    <row r="438">
+      <c r="A438" t="inlineStr">
+        <is>
+          <t>FR</t>
+        </is>
+      </c>
+      <c r="B438" t="inlineStr">
+        <is>
+          <t>unemployment_rate_25_74_total</t>
+        </is>
+      </c>
+      <c r="C438" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D438" t="n">
+        <v>7</v>
+      </c>
+      <c r="E438" t="n">
+        <v>6.4</v>
+      </c>
+      <c r="F438" t="inlineStr">
+        <is>
+          <t>PC_ACT</t>
+        </is>
+      </c>
+    </row>
+    <row r="439">
+      <c r="A439" t="inlineStr">
+        <is>
+          <t>FR</t>
+        </is>
+      </c>
+      <c r="B439" t="inlineStr">
+        <is>
+          <t>unemployment_rate_25_74_total</t>
+        </is>
+      </c>
+      <c r="C439" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D439" t="n">
+        <v>8</v>
+      </c>
+      <c r="E439" t="n">
+        <v>6.4</v>
+      </c>
+      <c r="F439" t="inlineStr">
+        <is>
+          <t>PC_ACT</t>
+        </is>
+      </c>
+    </row>
+    <row r="440">
+      <c r="A440" t="inlineStr">
+        <is>
+          <t>FR</t>
+        </is>
+      </c>
+      <c r="B440" t="inlineStr">
+        <is>
+          <t>unemployment_rate_25_74_total</t>
+        </is>
+      </c>
+      <c r="C440" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D440" t="n">
+        <v>9</v>
+      </c>
+      <c r="E440" t="n">
+        <v>6.4</v>
+      </c>
+      <c r="F440" t="inlineStr">
+        <is>
+          <t>PC_ACT</t>
+        </is>
+      </c>
+    </row>
+    <row r="441">
+      <c r="A441" t="inlineStr">
+        <is>
+          <t>FR</t>
+        </is>
+      </c>
+      <c r="B441" t="inlineStr">
+        <is>
+          <t>unemployment_rate_25_74_total</t>
+        </is>
+      </c>
+      <c r="C441" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D441" t="n">
+        <v>10</v>
+      </c>
+      <c r="E441" t="n">
+        <v>6.4</v>
+      </c>
+      <c r="F441" t="inlineStr">
+        <is>
+          <t>PC_ACT</t>
+        </is>
+      </c>
+    </row>
+    <row r="442">
+      <c r="A442" t="inlineStr">
+        <is>
+          <t>FR</t>
+        </is>
+      </c>
+      <c r="B442" t="inlineStr">
+        <is>
+          <t>unemployment_rate_25_74_total</t>
+        </is>
+      </c>
+      <c r="C442" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D442" t="n">
+        <v>11</v>
+      </c>
+      <c r="E442" t="n">
+        <v>6.4</v>
+      </c>
+      <c r="F442" t="inlineStr">
+        <is>
+          <t>PC_ACT</t>
+        </is>
+      </c>
+    </row>
+    <row r="443">
+      <c r="A443" t="inlineStr">
+        <is>
+          <t>FR</t>
+        </is>
+      </c>
+      <c r="B443" t="inlineStr">
+        <is>
+          <t>unemployment_rate_25_74_total</t>
+        </is>
+      </c>
+      <c r="C443" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D443" t="n">
+        <v>12</v>
+      </c>
+      <c r="E443" t="n">
+        <v>6.4</v>
+      </c>
+      <c r="F443" t="inlineStr">
+        <is>
+          <t>PC_ACT</t>
+        </is>
+      </c>
+    </row>
+    <row r="444">
+      <c r="A444" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="B444" t="inlineStr">
+        <is>
+          <t>unemployment_rate_25_74_total</t>
+        </is>
+      </c>
+      <c r="C444" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D444" t="n">
+        <v>2</v>
+      </c>
+      <c r="E444" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="F444" t="inlineStr">
+        <is>
+          <t>PC_ACT</t>
+        </is>
+      </c>
+    </row>
+    <row r="445">
+      <c r="A445" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="B445" t="inlineStr">
+        <is>
+          <t>unemployment_rate_25_74_total</t>
+        </is>
+      </c>
+      <c r="C445" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D445" t="n">
+        <v>3</v>
+      </c>
+      <c r="E445" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="F445" t="inlineStr">
+        <is>
+          <t>PC_ACT</t>
+        </is>
+      </c>
+    </row>
+    <row r="446">
+      <c r="A446" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="B446" t="inlineStr">
+        <is>
+          <t>unemployment_rate_25_74_total</t>
+        </is>
+      </c>
+      <c r="C446" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D446" t="n">
+        <v>4</v>
+      </c>
+      <c r="E446" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="F446" t="inlineStr">
+        <is>
+          <t>PC_ACT</t>
+        </is>
+      </c>
+    </row>
+    <row r="447">
+      <c r="A447" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="B447" t="inlineStr">
+        <is>
+          <t>unemployment_rate_25_74_total</t>
+        </is>
+      </c>
+      <c r="C447" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D447" t="n">
+        <v>5</v>
+      </c>
+      <c r="E447" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="F447" t="inlineStr">
+        <is>
+          <t>PC_ACT</t>
+        </is>
+      </c>
+    </row>
+    <row r="448">
+      <c r="A448" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="B448" t="inlineStr">
+        <is>
+          <t>unemployment_rate_25_74_total</t>
+        </is>
+      </c>
+      <c r="C448" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D448" t="n">
+        <v>6</v>
+      </c>
+      <c r="E448" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="F448" t="inlineStr">
+        <is>
+          <t>PC_ACT</t>
+        </is>
+      </c>
+    </row>
+    <row r="449">
+      <c r="A449" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="B449" t="inlineStr">
+        <is>
+          <t>unemployment_rate_25_74_total</t>
+        </is>
+      </c>
+      <c r="C449" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D449" t="n">
+        <v>7</v>
+      </c>
+      <c r="E449" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="F449" t="inlineStr">
+        <is>
+          <t>PC_ACT</t>
+        </is>
+      </c>
+    </row>
+    <row r="450">
+      <c r="A450" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="B450" t="inlineStr">
+        <is>
+          <t>unemployment_rate_25_74_total</t>
+        </is>
+      </c>
+      <c r="C450" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D450" t="n">
+        <v>8</v>
+      </c>
+      <c r="E450" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="F450" t="inlineStr">
+        <is>
+          <t>PC_ACT</t>
+        </is>
+      </c>
+    </row>
+    <row r="451">
+      <c r="A451" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="B451" t="inlineStr">
+        <is>
+          <t>unemployment_rate_25_74_total</t>
+        </is>
+      </c>
+      <c r="C451" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D451" t="n">
+        <v>9</v>
+      </c>
+      <c r="E451" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="F451" t="inlineStr">
+        <is>
+          <t>PC_ACT</t>
+        </is>
+      </c>
+    </row>
+    <row r="452">
+      <c r="A452" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="B452" t="inlineStr">
+        <is>
+          <t>unemployment_rate_25_74_total</t>
+        </is>
+      </c>
+      <c r="C452" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D452" t="n">
+        <v>10</v>
+      </c>
+      <c r="E452" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="F452" t="inlineStr">
+        <is>
+          <t>PC_ACT</t>
+        </is>
+      </c>
+    </row>
+    <row r="453">
+      <c r="A453" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="B453" t="inlineStr">
+        <is>
+          <t>unemployment_rate_25_74_total</t>
+        </is>
+      </c>
+      <c r="C453" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D453" t="n">
+        <v>11</v>
+      </c>
+      <c r="E453" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="F453" t="inlineStr">
+        <is>
+          <t>PC_ACT</t>
+        </is>
+      </c>
+    </row>
+    <row r="454">
+      <c r="A454" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="B454" t="inlineStr">
+        <is>
+          <t>unemployment_rate_25_74_total</t>
+        </is>
+      </c>
+      <c r="C454" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D454" t="n">
+        <v>12</v>
+      </c>
+      <c r="E454" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="F454" t="inlineStr">
+        <is>
+          <t>PC_ACT</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>geo</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>2025-02</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>2025-03</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>2025-04</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>2025-05</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>2025-06</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>2025-07</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>2025-08</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>2025-09</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>2025-10</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>2025-11</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>2025-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="C2" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="D2" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="E2" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="F2" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="G2" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="H2" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="I2" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="J2" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="K2" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="L2" t="n">
+        <v>3.5</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>9.6</v>
+      </c>
+      <c r="C3" t="n">
+        <v>9.6</v>
+      </c>
+      <c r="D3" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="E3" t="n">
+        <v>9.4</v>
+      </c>
+      <c r="F3" t="n">
+        <v>9.4</v>
+      </c>
+      <c r="G3" t="n">
+        <v>9.4</v>
+      </c>
+      <c r="H3" t="n">
+        <v>9.300000000000001</v>
+      </c>
+      <c r="I3" t="n">
+        <v>9.300000000000001</v>
+      </c>
+      <c r="J3" t="n">
+        <v>9.1</v>
+      </c>
+      <c r="K3" t="n">
+        <v>9.1</v>
+      </c>
+      <c r="L3" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>FR</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>6</v>
+      </c>
+      <c r="C4" t="n">
+        <v>6.2</v>
+      </c>
+      <c r="D4" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="E4" t="n">
+        <v>6.2</v>
+      </c>
+      <c r="F4" t="n">
+        <v>6.3</v>
+      </c>
+      <c r="G4" t="n">
+        <v>6.4</v>
+      </c>
+      <c r="H4" t="n">
+        <v>6.4</v>
+      </c>
+      <c r="I4" t="n">
+        <v>6.4</v>
+      </c>
+      <c r="J4" t="n">
+        <v>6.4</v>
+      </c>
+      <c r="K4" t="n">
+        <v>6.4</v>
+      </c>
+      <c r="L4" t="n">
+        <v>6.4</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>geo</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>2025-02</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>2025-03</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>2025-04</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>2025-05</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>2025-06</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>2025-07</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>2025-08</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>2025-09</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>2025-10</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>2025-11</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>2025-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>6.8</v>
+      </c>
+      <c r="C2" t="n">
+        <v>6.8</v>
+      </c>
+      <c r="D2" t="n">
+        <v>6.8</v>
+      </c>
+      <c r="E2" t="n">
+        <v>6.8</v>
+      </c>
+      <c r="F2" t="n">
+        <v>6.9</v>
+      </c>
+      <c r="G2" t="n">
+        <v>6.9</v>
+      </c>
+      <c r="H2" t="n">
+        <v>6.9</v>
+      </c>
+      <c r="I2" t="n">
+        <v>6.9</v>
+      </c>
+      <c r="J2" t="n">
+        <v>6.9</v>
+      </c>
+      <c r="K2" t="n">
+        <v>6.8</v>
+      </c>
+      <c r="L2" t="n">
+        <v>6.8</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>26.3</v>
+      </c>
+      <c r="C3" t="n">
+        <v>26.2</v>
+      </c>
+      <c r="D3" t="n">
+        <v>24.9</v>
+      </c>
+      <c r="E3" t="n">
+        <v>24.8</v>
+      </c>
+      <c r="F3" t="n">
+        <v>24.6</v>
+      </c>
+      <c r="G3" t="n">
+        <v>24.9</v>
+      </c>
+      <c r="H3" t="n">
+        <v>24.8</v>
+      </c>
+      <c r="I3" t="n">
+        <v>24.6</v>
+      </c>
+      <c r="J3" t="n">
+        <v>24.1</v>
+      </c>
+      <c r="K3" t="n">
+        <v>23.6</v>
+      </c>
+      <c r="L3" t="n">
+        <v>23.4</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>FR</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>19.8</v>
+      </c>
+      <c r="C4" t="n">
+        <v>19</v>
+      </c>
+      <c r="D4" t="n">
+        <v>18.9</v>
+      </c>
+      <c r="E4" t="n">
+        <v>19.1</v>
+      </c>
+      <c r="F4" t="n">
+        <v>18.8</v>
+      </c>
+      <c r="G4" t="n">
+        <v>18.5</v>
+      </c>
+      <c r="H4" t="n">
+        <v>18.6</v>
+      </c>
+      <c r="I4" t="n">
+        <v>19</v>
+      </c>
+      <c r="J4" t="n">
+        <v>18.9</v>
+      </c>
+      <c r="K4" t="n">
+        <v>18.5</v>
+      </c>
+      <c r="L4" t="n">
+        <v>18.1</v>
       </c>
     </row>
   </sheetData>
@@ -10732,7 +13491,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K4"/>
+  <dimension ref="A1:J4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10742,145 +13501,133 @@
         </is>
       </c>
       <c r="B1" t="n">
+        <v>2016</v>
+      </c>
+      <c r="C1" t="n">
+        <v>2017</v>
+      </c>
+      <c r="D1" t="n">
+        <v>2018</v>
+      </c>
+      <c r="E1" t="n">
+        <v>2019</v>
+      </c>
+      <c r="F1" t="n">
+        <v>2020</v>
+      </c>
+      <c r="G1" t="n">
         <v>2021</v>
       </c>
-      <c r="C1" t="n">
+      <c r="H1" t="n">
         <v>2022</v>
       </c>
-      <c r="D1" t="n">
+      <c r="I1" t="n">
         <v>2023</v>
       </c>
-      <c r="E1" t="n">
+      <c r="J1" t="n">
         <v>2024</v>
-      </c>
-      <c r="F1" t="n">
-        <v>2025</v>
-      </c>
-      <c r="G1" t="n">
-        <v>2026</v>
-      </c>
-      <c r="H1" t="n">
-        <v>2027</v>
-      </c>
-      <c r="I1" t="n">
-        <v>2028</v>
-      </c>
-      <c r="J1" t="n">
-        <v>2029</v>
-      </c>
-      <c r="K1" t="n">
-        <v>2030</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>DEU</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>5.5</v>
+        <v>30246.5082874666</v>
       </c>
       <c r="C2" t="n">
-        <v>10.8</v>
+        <v>31570.8974904355</v>
       </c>
       <c r="D2" t="n">
-        <v>3</v>
+        <v>33615.1802446285</v>
       </c>
       <c r="E2" t="n">
-        <v>2.5</v>
+        <v>35351.7793839047</v>
       </c>
       <c r="F2" t="n">
-        <v>1.7</v>
+        <v>36071.5163052037</v>
       </c>
       <c r="G2" t="n">
-        <v>1.9</v>
+        <v>37802.9092037468</v>
       </c>
       <c r="H2" t="n">
-        <v>2</v>
+        <v>42501.3770918378</v>
       </c>
       <c r="I2" t="n">
-        <v>2.1</v>
+        <v>45926.6267519884</v>
       </c>
       <c r="J2" t="n">
-        <v>2.2</v>
-      </c>
-      <c r="K2" t="n">
-        <v>2.2</v>
+        <v>47685.3791601533</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>ESP</t>
+          <t>ES</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>6.6</v>
+        <v>21291.8728491478</v>
       </c>
       <c r="C3" t="n">
-        <v>5.5</v>
+        <v>22141.1356335517</v>
       </c>
       <c r="D3" t="n">
-        <v>3.3</v>
+        <v>22663.3314861856</v>
       </c>
       <c r="E3" t="n">
-        <v>2.8</v>
+        <v>24582.9902204603</v>
       </c>
       <c r="F3" t="n">
-        <v>2.1</v>
+        <v>23782.4678049223</v>
       </c>
       <c r="G3" t="n">
-        <v>1.9</v>
+        <v>26175.863403135</v>
       </c>
       <c r="H3" t="n">
-        <v>2.5</v>
+        <v>28726.1264569898</v>
       </c>
       <c r="I3" t="n">
-        <v>2</v>
+        <v>33453.2943583124</v>
       </c>
       <c r="J3" t="n">
-        <v>2</v>
-      </c>
-      <c r="K3" t="n">
-        <v>2</v>
+        <v>35161.9297398487</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>FR</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>3.4</v>
+        <v>24924.9379154554</v>
       </c>
       <c r="C4" t="n">
-        <v>7</v>
+        <v>25436.327661389</v>
       </c>
       <c r="D4" t="n">
-        <v>4.2</v>
+        <v>26257.1585330353</v>
       </c>
       <c r="E4" t="n">
-        <v>1.7</v>
+        <v>28146.378960002</v>
       </c>
       <c r="F4" t="n">
-        <v>1.5</v>
+        <v>28877.5207135287</v>
       </c>
       <c r="G4" t="n">
-        <v>1.1</v>
+        <v>30167.6571699568</v>
       </c>
       <c r="H4" t="n">
-        <v>2.5</v>
+        <v>33737.7298976999</v>
       </c>
       <c r="I4" t="n">
-        <v>1.4</v>
+        <v>37582.228371007</v>
       </c>
       <c r="J4" t="n">
-        <v>2.7</v>
-      </c>
-      <c r="K4" t="n">
-        <v>0.8</v>
+        <v>39420.8018012013</v>
       </c>
     </row>
   </sheetData>
@@ -10941,34 +13688,34 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>81.995</v>
+        <v>5.5</v>
       </c>
       <c r="C2" t="n">
-        <v>82.529</v>
+        <v>10.8</v>
       </c>
       <c r="D2" t="n">
-        <v>83.28700000000001</v>
+        <v>3</v>
       </c>
       <c r="E2" t="n">
-        <v>83.517</v>
+        <v>2.5</v>
       </c>
       <c r="F2" t="n">
-        <v>83.664</v>
+        <v>1.7</v>
       </c>
       <c r="G2" t="n">
-        <v>83.777</v>
+        <v>1.9</v>
       </c>
       <c r="H2" t="n">
-        <v>83.845</v>
+        <v>2</v>
       </c>
       <c r="I2" t="n">
-        <v>83.874</v>
+        <v>2.1</v>
       </c>
       <c r="J2" t="n">
-        <v>83.89100000000001</v>
+        <v>2.2</v>
       </c>
       <c r="K2" t="n">
-        <v>83.893</v>
+        <v>2.2</v>
       </c>
     </row>
     <row r="3">
@@ -10978,34 +13725,34 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>47.487</v>
+        <v>6.6</v>
       </c>
       <c r="C3" t="n">
-        <v>48.085</v>
+        <v>5.5</v>
       </c>
       <c r="D3" t="n">
-        <v>48.628</v>
+        <v>3.3</v>
       </c>
       <c r="E3" t="n">
-        <v>49.078</v>
+        <v>2.8</v>
       </c>
       <c r="F3" t="n">
-        <v>49.721</v>
+        <v>2.1</v>
       </c>
       <c r="G3" t="n">
-        <v>50.314</v>
+        <v>1.9</v>
       </c>
       <c r="H3" t="n">
-        <v>50.84</v>
+        <v>2.5</v>
       </c>
       <c r="I3" t="n">
-        <v>51.294</v>
+        <v>2</v>
       </c>
       <c r="J3" t="n">
-        <v>51.679</v>
+        <v>2</v>
       </c>
       <c r="K3" t="n">
-        <v>52.004</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4">
@@ -11015,34 +13762,34 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>67.697</v>
+        <v>3.4</v>
       </c>
       <c r="C4" t="n">
-        <v>68.06</v>
+        <v>7</v>
       </c>
       <c r="D4" t="n">
-        <v>68.246</v>
+        <v>4.2</v>
       </c>
       <c r="E4" t="n">
-        <v>68.437</v>
+        <v>1.7</v>
       </c>
       <c r="F4" t="n">
-        <v>68.628</v>
+        <v>1.5</v>
       </c>
       <c r="G4" t="n">
-        <v>68.821</v>
+        <v>1.1</v>
       </c>
       <c r="H4" t="n">
-        <v>69.014</v>
+        <v>2.5</v>
       </c>
       <c r="I4" t="n">
-        <v>69.20699999999999</v>
+        <v>1.4</v>
       </c>
       <c r="J4" t="n">
-        <v>69.401</v>
+        <v>2.7</v>
       </c>
       <c r="K4" t="n">
-        <v>69.596</v>
+        <v>0.8</v>
       </c>
     </row>
   </sheetData>
@@ -11103,34 +13850,34 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>3.9</v>
+        <v>81.995</v>
       </c>
       <c r="C2" t="n">
-        <v>1.8</v>
+        <v>82.529</v>
       </c>
       <c r="D2" t="n">
-        <v>-0.9</v>
+        <v>83.28700000000001</v>
       </c>
       <c r="E2" t="n">
-        <v>-0.5</v>
+        <v>83.517</v>
       </c>
       <c r="F2" t="n">
-        <v>0.2</v>
+        <v>83.664</v>
       </c>
       <c r="G2" t="n">
-        <v>0.9</v>
+        <v>83.777</v>
       </c>
       <c r="H2" t="n">
-        <v>1.5</v>
+        <v>83.845</v>
       </c>
       <c r="I2" t="n">
-        <v>1.2</v>
+        <v>83.874</v>
       </c>
       <c r="J2" t="n">
-        <v>1</v>
+        <v>83.89100000000001</v>
       </c>
       <c r="K2" t="n">
-        <v>0.7</v>
+        <v>83.893</v>
       </c>
     </row>
     <row r="3">
@@ -11140,34 +13887,34 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>6.7</v>
+        <v>47.487</v>
       </c>
       <c r="C3" t="n">
-        <v>6.4</v>
+        <v>48.085</v>
       </c>
       <c r="D3" t="n">
-        <v>2.5</v>
+        <v>48.628</v>
       </c>
       <c r="E3" t="n">
-        <v>3.5</v>
+        <v>49.078</v>
       </c>
       <c r="F3" t="n">
-        <v>2.9</v>
+        <v>49.721</v>
       </c>
       <c r="G3" t="n">
-        <v>2</v>
+        <v>50.314</v>
       </c>
       <c r="H3" t="n">
-        <v>1.7</v>
+        <v>50.84</v>
       </c>
       <c r="I3" t="n">
-        <v>1.6</v>
+        <v>51.294</v>
       </c>
       <c r="J3" t="n">
-        <v>1.6</v>
+        <v>51.679</v>
       </c>
       <c r="K3" t="n">
-        <v>1.6</v>
+        <v>52.004</v>
       </c>
     </row>
     <row r="4">
@@ -11177,34 +13924,34 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>6.8</v>
+        <v>67.697</v>
       </c>
       <c r="C4" t="n">
-        <v>2.8</v>
+        <v>68.06</v>
       </c>
       <c r="D4" t="n">
-        <v>1.6</v>
+        <v>68.246</v>
       </c>
       <c r="E4" t="n">
-        <v>1.1</v>
+        <v>68.437</v>
       </c>
       <c r="F4" t="n">
-        <v>0.7</v>
+        <v>68.628</v>
       </c>
       <c r="G4" t="n">
-        <v>0.9</v>
+        <v>68.821</v>
       </c>
       <c r="H4" t="n">
-        <v>1.2</v>
+        <v>69.014</v>
       </c>
       <c r="I4" t="n">
-        <v>1.3</v>
+        <v>69.20699999999999</v>
       </c>
       <c r="J4" t="n">
-        <v>1.2</v>
+        <v>69.401</v>
       </c>
       <c r="K4" t="n">
-        <v>1.2</v>
+        <v>69.596</v>
       </c>
     </row>
   </sheetData>
@@ -11218,6 +13965,168 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:K4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>geo</t>
+        </is>
+      </c>
+      <c r="B1" t="n">
+        <v>2021</v>
+      </c>
+      <c r="C1" t="n">
+        <v>2022</v>
+      </c>
+      <c r="D1" t="n">
+        <v>2023</v>
+      </c>
+      <c r="E1" t="n">
+        <v>2024</v>
+      </c>
+      <c r="F1" t="n">
+        <v>2025</v>
+      </c>
+      <c r="G1" t="n">
+        <v>2026</v>
+      </c>
+      <c r="H1" t="n">
+        <v>2027</v>
+      </c>
+      <c r="I1" t="n">
+        <v>2028</v>
+      </c>
+      <c r="J1" t="n">
+        <v>2029</v>
+      </c>
+      <c r="K1" t="n">
+        <v>2030</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>DEU</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>3.9</v>
+      </c>
+      <c r="C2" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="D2" t="n">
+        <v>-0.9</v>
+      </c>
+      <c r="E2" t="n">
+        <v>-0.5</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="H2" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="I2" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="J2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K2" t="n">
+        <v>0.7</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>ESP</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>6.7</v>
+      </c>
+      <c r="C3" t="n">
+        <v>6.4</v>
+      </c>
+      <c r="D3" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="E3" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="F3" t="n">
+        <v>2.9</v>
+      </c>
+      <c r="G3" t="n">
+        <v>2</v>
+      </c>
+      <c r="H3" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="I3" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="J3" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="K3" t="n">
+        <v>1.6</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>FRA</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>6.8</v>
+      </c>
+      <c r="C4" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="D4" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="E4" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="H4" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="I4" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="J4" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="K4" t="n">
+        <v>1.2</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:F4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>

</xml_diff>